<commit_message>
mejoras del dia miercoles 22 de julio  primer commit del dia
</commit_message>
<xml_diff>
--- a/app/lib/plantillas-costeo/tabla-costeo-v3.xlsx
+++ b/app/lib/plantillas-costeo/tabla-costeo-v3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\droku\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF7729B5-7E50-4CD3-B0F4-6B771AF29AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F875443-1EDB-4A89-ACF2-F65A37A493ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Costeo" sheetId="1" r:id="rId1"/>
@@ -2042,7 +2042,9 @@
       <c r="E4" s="21">
         <v>1</v>
       </c>
-      <c r="F4" s="22"/>
+      <c r="F4" s="22">
+        <v>0</v>
+      </c>
       <c r="G4" s="23">
         <f t="shared" ref="G4:G23" si="0">F4/1.19</f>
         <v>0</v>
@@ -2105,7 +2107,7 @@
       <c r="E5" s="21">
         <v>1</v>
       </c>
-      <c r="F5" s="35">
+      <c r="F5" s="22">
         <v>0</v>
       </c>
       <c r="G5" s="23">
@@ -3338,7 +3340,7 @@
       </c>
       <c r="F24" s="18" t="b">
         <f>K24&lt;K26</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" s="44"/>
       <c r="H24" s="24">
@@ -3430,7 +3432,7 @@
       </c>
       <c r="K26" s="56">
         <f>F27/1.19</f>
-        <v>0</v>
+        <v>4201680.6722689075</v>
       </c>
       <c r="L26" s="53"/>
       <c r="M26" s="2"/>
@@ -3459,7 +3461,9 @@
         <v>50</v>
       </c>
       <c r="E27" s="108"/>
-      <c r="F27" s="58"/>
+      <c r="F27" s="58">
+        <v>5000000</v>
+      </c>
       <c r="G27" s="2"/>
       <c r="H27" s="59"/>
       <c r="I27" s="2"/>
@@ -3628,16 +3632,16 @@
         <v>58</v>
       </c>
       <c r="K31" s="68" t="e">
-        <f>1-(J29/J28)</f>
-        <v>#VALUE!</v>
+        <f>1-(K29/K28)</f>
+        <v>#DIV/0!</v>
       </c>
       <c r="L31" s="53"/>
       <c r="M31" s="3" t="s">
         <v>58</v>
       </c>
       <c r="N31" s="68" t="e">
-        <f>1-(M29/M28)</f>
-        <v>#VALUE!</v>
+        <f>1-(N29/N28)</f>
+        <v>#DIV/0!</v>
       </c>
       <c r="P31" s="2"/>
       <c r="Q31" s="2"/>
@@ -3667,9 +3671,9 @@
       <c r="J32" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="K32" s="68" t="e">
-        <f>1-(J28/J26)</f>
-        <v>#VALUE!</v>
+      <c r="K32" s="68">
+        <f>1-(K28/K26)</f>
+        <v>1</v>
       </c>
       <c r="L32" s="53"/>
       <c r="M32" s="2" t="s">

</xml_diff>